<commit_message>
feat(investor): mise a jour portefeuille VOLTA a 14.50 MW (29 stations) et nouvelles metriques financieres de l'etude certifiee
</commit_message>
<xml_diff>
--- a/public/documents/dataroom/Hypotheses_revenus_FCR_aFRR_MdC_VOLTA.xlsx
+++ b/public/documents/dataroom/Hypotheses_revenus_FCR_aFRR_MdC_VOLTA.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Synthese BESS Volta" sheetId="1" r:id="rId1"/>
-    <sheet name="Detail 31 Stations BESS" sheetId="2" r:id="rId2"/>
+    <sheet name="Detail 29 Stations BESS" sheetId="2" r:id="rId2"/>
     <sheet name="Chiffrage TURPE 7" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,12 +399,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D27"/>
   <cols>
-    <col min="1" max="1" width="48.83203125" customWidth="1"/>
+    <col min="1" max="1" width="50.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,7 +417,7 @@
         <v>Type d'actif</v>
       </c>
       <c r="B2" t="str">
-        <v>Stations de Stockage par Batterie Décentralisées BESS (LiFePO4 / NMC)</v>
+        <v>Stations de Stockage par Batterie Décentralisées BESS (CESC Mercury 261 / LiFePO4)</v>
       </c>
     </row>
     <row r="3">
@@ -425,275 +425,311 @@
         <v>Nombre de stations</v>
       </c>
       <c r="B3">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Puissance unitaire par station</v>
-      </c>
-      <c r="B4" t="str">
-        <v>500 kW / 1 000 kWh (1 MWh)</v>
+        <v>Nombre de projets fonciers</v>
+      </c>
+      <c r="B4">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Puissance totale raccordée</v>
+        <v>Puissance unitaire par station</v>
       </c>
       <c r="B5" t="str">
-        <v>15 500 kW (15.5 MW)</v>
+        <v>500 kW / 1 044 kWh</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Capacité totale de stockage</v>
+        <v>Puissance totale raccordée</v>
       </c>
       <c r="B6" t="str">
-        <v>31 000 kWh (31 MWh)</v>
+        <v>14 500 kW (14.50 MW)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Mode de fonctionnement</v>
+        <v>Capacité totale de stockage</v>
       </c>
       <c r="B7" t="str">
-        <v>2 cycles complets quotidiens (Charge nuit/midi, Décharge matin/soir)</v>
+        <v>30 276 kWh (30.28 MWh)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Mode de fonctionnement</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2 cycles complets quotidiens (Value Stacking 24h/24)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>Date d'audit de référence</v>
       </c>
-      <c r="B8" t="str">
-        <v>30 Septembre 2026</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>INDICATEURS CLÉS DE PERFORMANCE (KPIs CONSOLIDÉS)</v>
-      </c>
-      <c r="B10" t="str">
-        <v>VALEUR</v>
-      </c>
-      <c r="C10" t="str">
-        <v>UNITÉ / BASE</v>
-      </c>
-      <c r="D10" t="str">
-        <v>SOURCES / MARCHÉS</v>
+      <c r="B9" t="str">
+        <v>06 Octobre 2026</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Chiffre d'Affaires Brut Annuel Consolidé</v>
-      </c>
-      <c r="B11">
-        <v>2860000</v>
+        <v>INDICATEURS CLÉS DE PERFORMANCE (KPIs CONSOLIDÉS)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>VALEUR</v>
       </c>
       <c r="C11" t="str">
-        <v>€ HT / an</v>
+        <v>UNITÉ / BASE</v>
       </c>
       <c r="D11" t="str">
-        <v>2 cycles/jour multi-marchés</v>
+        <v>SOURCES / MARCHÉS</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>1. Réserve Primaire de Fréquence (FCR) &amp; PICASSO</v>
+        <v>Chiffre d'Affaires Brut Annuel Consolidé (An 1)</v>
       </c>
       <c r="B12">
-        <v>2076882</v>
+        <v>2701952</v>
       </c>
       <c r="C12" t="str">
-        <v>€ HT / an (72%)</v>
+        <v>€ HT / an</v>
       </c>
       <c r="D12" t="str">
-        <v>Adjudications journalières RTE</v>
+        <v>Value Stacking 29 stations (2 cycles/j)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2. Arbitrage SPOT (Day-Ahead &amp; Intraday EPEX SPOT)</v>
+        <v>1. Réserve Primaire 50 Hz (FCR) &amp; PICASSO (aFRR)</v>
       </c>
       <c r="B13">
-        <v>504780</v>
+        <v>1584144</v>
       </c>
       <c r="C13" t="str">
-        <v>€ HT / an (18%)</v>
+        <v>€ HT / an (58.7%)</v>
       </c>
       <c r="D13" t="str">
-        <v>Spreads horaires de prix électricité</v>
+        <v>Rémunération puissance symétrique RTE/PICASSO</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>3. Marché de Capacité (PP2)</v>
+        <v>2. Arbitrage SPOT (Day-Ahead &amp; Intraday EPEX SPOT)</v>
       </c>
       <c r="B14">
-        <v>271253</v>
+        <v>884065</v>
       </c>
       <c r="C14" t="str">
-        <v>€ HT / an (10%)</v>
+        <v>€ HT / an (31.8%)</v>
       </c>
       <c r="D14" t="str">
-        <v>Disponibilité heures de pointe hivernales</v>
+        <v>Spreads horaires 2 cycles/jour (Creux/Pointes)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Gain Réforme Réglementaire TURPE 7 (CRE 2025-227)</v>
+        <v>3. Marché de Capacité RTE (PP2 Hiver)</v>
       </c>
       <c r="B15">
-        <v>439073</v>
+        <v>253750</v>
       </c>
       <c r="C15" t="str">
-        <v>€ HT / an net</v>
+        <v>€ HT / an (9.5%)</v>
       </c>
       <c r="D15" t="str">
-        <v>Exonération &gt;80% de la double taxation</v>
+        <v>Garantie de puissance 35 €/kW/an (derating 0.5)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Facture Réseau Révisée sous TURPE 7</v>
+        <v>Gain Réforme Réglementaire TURPE 7 (CRE 2025-227)</v>
       </c>
       <c r="B16">
-        <v>257627</v>
+        <v>411307</v>
       </c>
       <c r="C16" t="str">
-        <v>€ / an vs 697 586 €</v>
+        <v>€ HT / an net</v>
       </c>
       <c r="D16" t="str">
-        <v>-63% de baisse des coûts d'accès réseau</v>
+        <v>Exonération &gt;80% soutirage/injection</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>OPEX annuel d'exploitation consolidé</v>
+        <v>Facture Réseau Révisée sous TURPE 7</v>
       </c>
       <c r="B17">
-        <v>-1140000</v>
+        <v>241127</v>
       </c>
       <c r="C17" t="str">
-        <v>€ HT / an</v>
+        <v>€ / an vs 652 434 €</v>
       </c>
       <c r="D17" t="str">
-        <v>Maintenance constructeur, assurance, loyers dalles</v>
+        <v>-63% de baisse des coûts d'accès réseau</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>EBITDA Net d'Exploitation Annuel</v>
+        <v>OPEX annuel d'exploitation consolidé (An 1)</v>
       </c>
       <c r="B18">
-        <v>1720000</v>
+        <v>-1077101</v>
       </c>
       <c r="C18" t="str">
         <v>€ HT / an</v>
       </c>
       <c r="D18" t="str">
-        <v>Marge opérationnelle nette &gt; 60%</v>
+        <v>Maintenance constructeur, assurance, loyers baux 20 ans</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CAPEX Global 31 Stations Clé en Main</v>
+        <v>EBITDA Net d'Exploitation Annuel (An 1)</v>
       </c>
       <c r="B19">
-        <v>10850000</v>
+        <v>1624851</v>
       </c>
       <c r="C19" t="str">
-        <v>€ HT</v>
+        <v>€ HT / an</v>
       </c>
       <c r="D19" t="str">
-        <v>~350 k€ / station de 1 MWh raccordée HTA</v>
+        <v>Marge opérationnelle nette ~60%</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>TRI Projet (IRR avant financement)</v>
-      </c>
-      <c r="B20" t="str">
-        <v>20.5%</v>
+        <v>CAPEX Global 29 Stations Clé en Main</v>
+      </c>
+      <c r="B20">
+        <v>8400000</v>
       </c>
       <c r="C20" t="str">
-        <v>Pourcentage</v>
+        <v>€ HT</v>
       </c>
       <c r="D20" t="str">
-        <v>Sur horizon d'exploitation 15 ans</v>
+        <v>~290 k€ / station de 500 kW raccordée HTA</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>TRI Fonds Propres (Equity IRR)</v>
-      </c>
-      <c r="B21" t="str">
-        <v>37.4%</v>
+        <v>Service de la dette senior (12 ans @ 4.30%)</v>
+      </c>
+      <c r="B21">
+        <v>-910519</v>
       </c>
       <c r="C21" t="str">
-        <v>Pourcentage</v>
+        <v>€ / an</v>
       </c>
       <c r="D21" t="str">
-        <v>Effet de levier bancaire optimisé</v>
+        <v>Amortissement constant sur 12 ans</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Ratio de couverture bancaire DSCR</v>
-      </c>
-      <c r="B22" t="str">
-        <v>2.34x</v>
+        <v>Cash-Flow Net Annuel An 1 (Post-dette)</v>
+      </c>
+      <c r="B22">
+        <v>714332</v>
       </c>
       <c r="C22" t="str">
-        <v>Ratio moyen</v>
+        <v>€ / an</v>
       </c>
       <c r="D22" t="str">
-        <v>Classement bancabilité très élevé</v>
+        <v>Trésorerie nette disponible An 1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Temps de retour sur Fonds Propres (Payback)</v>
-      </c>
-      <c r="B23">
-        <v>2.2</v>
+        <v>TRI Projet (IRR avant financement)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>20.5%</v>
       </c>
       <c r="C23" t="str">
-        <v>Années</v>
+        <v>Pourcentage</v>
       </c>
       <c r="D23" t="str">
-        <v>Rentabilité accélérée</v>
+        <v>Sur horizon d'exploitation 15 ans</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>TRI Fonds Propres (Equity IRR)</v>
+      </c>
+      <c r="B24" t="str">
+        <v>37.4%</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Pourcentage</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Effet de levier bancaire optimisé</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Ratio de couverture bancaire DSCR</v>
+      </c>
+      <c r="B25" t="str">
+        <v>1.91x</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Ratio moyen</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Classement bancabilité très élevé (Seuil &gt; 1.50x)</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Temps de retour sur Fonds Propres (Payback)</v>
+      </c>
+      <c r="B26">
+        <v>2.2</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Années</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Rentabilité accélérée</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>Temps de retour Projet global</v>
       </c>
-      <c r="B24">
-        <v>4.6</v>
-      </c>
-      <c r="C24" t="str">
+      <c r="B27">
+        <v>5</v>
+      </c>
+      <c r="C27" t="str">
         <v>Années</v>
       </c>
-      <c r="D24" t="str">
-        <v>Seuil cible &lt; 5 ans</v>
+      <c r="D27" t="str">
+        <v>Amortissement complet du CAPEX</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D27"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L31"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="6.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="18.83203125" customWidth="1"/>
     <col min="8" max="8" width="22.83203125" customWidth="1"/>
@@ -707,7 +743,7 @@
         <v>N° Station</v>
       </c>
       <c r="B1" t="str">
-        <v>Nom du Site</v>
+        <v>Nom du Site / Projet</v>
       </c>
       <c r="C1" t="str">
         <v>Commune / CP</v>
@@ -745,7 +781,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>BRANTÔME</v>
+        <v>BRANTÔME EN PÉRIGORD</v>
       </c>
       <c r="C2" t="str">
         <v>24310 BRANTÔME</v>
@@ -763,7 +799,7 @@
         <v>1044</v>
       </c>
       <c r="H2">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I2" t="str">
         <v>BRANTOME (3.5 km)</v>
@@ -801,7 +837,7 @@
         <v>1044</v>
       </c>
       <c r="H3">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I3" t="str">
         <v>PLAUD (6.6 km)</v>
@@ -839,7 +875,7 @@
         <v>1044</v>
       </c>
       <c r="H4">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I4" t="str">
         <v>SEMEZIES (5.9 km)</v>
@@ -877,7 +913,7 @@
         <v>1044</v>
       </c>
       <c r="H5">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I5" t="str">
         <v>LE REPAIRE (8.6 km)</v>
@@ -915,7 +951,7 @@
         <v>1044</v>
       </c>
       <c r="H6">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I6" t="str">
         <v>LUBERSAC (8.3 km)</v>
@@ -953,7 +989,7 @@
         <v>1044</v>
       </c>
       <c r="H7">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I7" t="str">
         <v>GUICHE (4.9 km)</v>
@@ -991,7 +1027,7 @@
         <v>1044</v>
       </c>
       <c r="H8">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I8" t="str">
         <v>LESQUIVE 2 (2.3 km)</v>
@@ -1029,7 +1065,7 @@
         <v>1044</v>
       </c>
       <c r="H9">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I9" t="str">
         <v>LUBERSAC (8.6 km)</v>
@@ -1049,7 +1085,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>SAINT-ÉLOY-LES-TUILERIES</v>
+        <v>SAINT-ÉLOY-LES-TUILERIES (GRANGER)</v>
       </c>
       <c r="C10" t="str">
         <v>19210 ST-ELOY</v>
@@ -1067,7 +1103,7 @@
         <v>1044</v>
       </c>
       <c r="H10">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I10" t="str">
         <v>LUBERSAC (10.5 km)</v>
@@ -1105,7 +1141,7 @@
         <v>1044</v>
       </c>
       <c r="H11">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I11" t="str">
         <v>LERE (5.7 km)</v>
@@ -1143,7 +1179,7 @@
         <v>1044</v>
       </c>
       <c r="H12">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I12" t="str">
         <v>LERE (5.7 km)</v>
@@ -1181,7 +1217,7 @@
         <v>1044</v>
       </c>
       <c r="H13">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I13" t="str">
         <v>LERE (3.6 km)</v>
@@ -1219,7 +1255,7 @@
         <v>1044</v>
       </c>
       <c r="H14">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I14" t="str">
         <v>LERE (6.2 km)</v>
@@ -1257,7 +1293,7 @@
         <v>1044</v>
       </c>
       <c r="H15">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I15" t="str">
         <v>STE-FOY (9.0 km)</v>
@@ -1295,7 +1331,7 @@
         <v>1044</v>
       </c>
       <c r="H16">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I16" t="str">
         <v>BOUSSAC (5.9 km)</v>
@@ -1333,7 +1369,7 @@
         <v>1044</v>
       </c>
       <c r="H17">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I17" t="str">
         <v>LA SAUVETAT (11.8 km)</v>
@@ -1371,7 +1407,7 @@
         <v>1044</v>
       </c>
       <c r="H18">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I18" t="str">
         <v>NONTRON (13.7 km)</v>
@@ -1409,7 +1445,7 @@
         <v>1044</v>
       </c>
       <c r="H19">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I19" t="str">
         <v>CHATELUS 2 (5.4 km)</v>
@@ -1447,7 +1483,7 @@
         <v>1044</v>
       </c>
       <c r="H20">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I20" t="str">
         <v>ETAULIERS (7.7 km)</v>
@@ -1485,7 +1521,7 @@
         <v>1044</v>
       </c>
       <c r="H21">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I21" t="str">
         <v>LUBERSAC (6.9 km)</v>
@@ -1523,7 +1559,7 @@
         <v>1044</v>
       </c>
       <c r="H22">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I22" t="str">
         <v>AURIOLLES (7.9 km)</v>
@@ -1561,7 +1597,7 @@
         <v>1044</v>
       </c>
       <c r="H23">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I23" t="str">
         <v>VIC-EN-BIGORRE (10.8 km)</v>
@@ -1581,16 +1617,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>MAISONNISSES</v>
+        <v>SAINT EUTROPE DE BORN</v>
       </c>
       <c r="C24" t="str">
-        <v>23150 MAISONNISSES</v>
+        <v>47210 ST-EUTROPE</v>
       </c>
       <c r="D24" t="str">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="E24" t="str">
-        <v>LARDY Christian</v>
+        <v>FRECHEVILLE Mathieu</v>
       </c>
       <c r="F24">
         <v>500</v>
@@ -1599,10 +1635,10 @@
         <v>1044</v>
       </c>
       <c r="H24">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I24" t="str">
-        <v>LAVAUD (10.6 km)</v>
+        <v>CANCON (7.2 km)</v>
       </c>
       <c r="J24">
         <v>3000</v>
@@ -1619,16 +1655,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>SAINT EUTROPE DE BORN</v>
+        <v>BEYCHAC-ET-CAILLAU</v>
       </c>
       <c r="C25" t="str">
-        <v>47210 ST-EUTROPE</v>
+        <v>33750 BEYCHAC</v>
       </c>
       <c r="D25" t="str">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E25" t="str">
-        <v>FRECHEVILLE Mathieu</v>
+        <v>DOUMENS Jacques</v>
       </c>
       <c r="F25">
         <v>500</v>
@@ -1637,10 +1673,10 @@
         <v>1044</v>
       </c>
       <c r="H25">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I25" t="str">
-        <v>CANCON (7.2 km)</v>
+        <v>POMPIGNAC (4.0 km)</v>
       </c>
       <c r="J25">
         <v>3000</v>
@@ -1657,16 +1693,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>BEYCHAC-ET-CAILLAU</v>
+        <v>VENDAYS-MONTALIVET</v>
       </c>
       <c r="C26" t="str">
-        <v>33750 BEYCHAC</v>
+        <v>33930 VENDAYS</v>
       </c>
       <c r="D26" t="str">
         <v>33</v>
       </c>
       <c r="E26" t="str">
-        <v>DOUMENS Jacques</v>
+        <v>HOUSSAIT-YOUNG Paul</v>
       </c>
       <c r="F26">
         <v>500</v>
@@ -1675,10 +1711,10 @@
         <v>1044</v>
       </c>
       <c r="H26">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I26" t="str">
-        <v>POMPIGNAC (4.0 km)</v>
+        <v>ST-VIVIEN (9.9 km)</v>
       </c>
       <c r="J26">
         <v>3000</v>
@@ -1695,16 +1731,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>VENDAYS-MONTALIVET</v>
+        <v>SAINT-MARTIN-DE-FRESSENGEAS</v>
       </c>
       <c r="C27" t="str">
-        <v>33930 VENDAYS</v>
+        <v>24800 ST-MARTIN</v>
       </c>
       <c r="D27" t="str">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E27" t="str">
-        <v>HOUSSAIT-YOUNG Paul</v>
+        <v>MISSAULT Cécile</v>
       </c>
       <c r="F27">
         <v>500</v>
@@ -1713,10 +1749,10 @@
         <v>1044</v>
       </c>
       <c r="H27">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I27" t="str">
-        <v>ST-VIVIEN (9.9 km)</v>
+        <v>THIVIERS (6.7 km)</v>
       </c>
       <c r="J27">
         <v>3000</v>
@@ -1733,16 +1769,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>SAINT-MARTIN-DE-FRESSENGEAS</v>
+        <v>MOURIOUX-VIEILLEVILLE 2</v>
       </c>
       <c r="C28" t="str">
-        <v>24800 ST-MARTIN</v>
+        <v>23210 MOURIOUX</v>
       </c>
       <c r="D28" t="str">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E28" t="str">
-        <v>MISSAULT Cécile</v>
+        <v>MEILLAT Patrick</v>
       </c>
       <c r="F28">
         <v>500</v>
@@ -1751,10 +1787,10 @@
         <v>1044</v>
       </c>
       <c r="H28">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I28" t="str">
-        <v>THIVIERS (6.7 km)</v>
+        <v>CHATELUS 2 (5.4 km)</v>
       </c>
       <c r="J28">
         <v>3000</v>
@@ -1771,16 +1807,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>BEYSSENAC</v>
+        <v>ARGENCES EN AUBRAC</v>
       </c>
       <c r="C29" t="str">
-        <v>19230 BEYSSENAC</v>
+        <v>12420 ARGENCES</v>
       </c>
       <c r="D29" t="str">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E29" t="str">
-        <v>CELERIE Guy</v>
+        <v>DOMERGUE Daniel</v>
       </c>
       <c r="F29">
         <v>500</v>
@@ -1789,10 +1825,10 @@
         <v>1044</v>
       </c>
       <c r="H29">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I29" t="str">
-        <v>LUBERSAC (7.1 km)</v>
+        <v>RUEYRES (5.9 km)</v>
       </c>
       <c r="J29">
         <v>3000</v>
@@ -1809,16 +1845,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>MOURIOUX-VIEILLEVILLE 2</v>
+        <v>SAINT-ÉLOY-LES-TUILERIES (COMBY)</v>
       </c>
       <c r="C30" t="str">
-        <v>23210 MOURIOUX</v>
+        <v>19210 ST-ELOY</v>
       </c>
       <c r="D30" t="str">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E30" t="str">
-        <v>MEILLAT Patrick</v>
+        <v>COMBY Fabrice</v>
       </c>
       <c r="F30">
         <v>500</v>
@@ -1827,10 +1863,10 @@
         <v>1044</v>
       </c>
       <c r="H30">
-        <v>32</v>
+        <v>19.84</v>
       </c>
       <c r="I30" t="str">
-        <v>CHATELUS 2 (5.4 km)</v>
+        <v>LUBERSAC (8.3 km)</v>
       </c>
       <c r="J30">
         <v>3000</v>
@@ -1843,122 +1879,46 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31">
-        <v>30</v>
+      <c r="A31" t="str">
+        <v>TOTAL</v>
       </c>
       <c r="B31" t="str">
-        <v>ARGENCES EN AUBRAC</v>
+        <v>29 STATIONS BESS (26 PROJETS DONT CLUSTER CASTEBRUNET)</v>
       </c>
       <c r="C31" t="str">
-        <v>12420 ARGENCES</v>
+        <v>AQUITAINE / OCCITANIE</v>
       </c>
       <c r="D31" t="str">
-        <v>12</v>
+        <v>8 Dpts</v>
       </c>
       <c r="E31" t="str">
-        <v>DOMERGUE Daniel</v>
+        <v>26 Bailleurs notariés</v>
       </c>
       <c r="F31">
-        <v>500</v>
+        <v>14500</v>
       </c>
       <c r="G31">
-        <v>1044</v>
+        <v>30276</v>
       </c>
       <c r="H31">
-        <v>32</v>
+        <v>575.36</v>
       </c>
       <c r="I31" t="str">
-        <v>RUEYRES (5.9 km)</v>
+        <v>26 Postes sources</v>
       </c>
       <c r="J31">
-        <v>3000</v>
+        <v>87000</v>
       </c>
       <c r="K31" t="str">
-        <v>PdB signée 20 ans</v>
+        <v>100% Sécurisé</v>
       </c>
       <c r="L31" t="str">
-        <v>URBA OK</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" t="str">
-        <v>SAINT-ÉLOY-LES-TUILERIES (COMBY)</v>
-      </c>
-      <c r="C32" t="str">
-        <v>19210 ST-ELOY</v>
-      </c>
-      <c r="D32" t="str">
-        <v>19</v>
-      </c>
-      <c r="E32" t="str">
-        <v>COMBY Fabrice</v>
-      </c>
-      <c r="F32">
-        <v>500</v>
-      </c>
-      <c r="G32">
-        <v>1044</v>
-      </c>
-      <c r="H32">
-        <v>32</v>
-      </c>
-      <c r="I32" t="str">
-        <v>LUBERSAC (8.3 km)</v>
-      </c>
-      <c r="J32">
-        <v>3000</v>
-      </c>
-      <c r="K32" t="str">
-        <v>PdB signée 20 ans</v>
-      </c>
-      <c r="L32" t="str">
-        <v>URBA OK</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B33" t="str">
-        <v>31 STATIONS BESS (28 PROJETS DONT CLUSTER CASTEBRUNET)</v>
-      </c>
-      <c r="C33" t="str">
-        <v>AQUITAINE / OCCITANIE</v>
-      </c>
-      <c r="D33" t="str">
-        <v>8 Dpts</v>
-      </c>
-      <c r="E33" t="str">
-        <v>28 Bailleurs notariés</v>
-      </c>
-      <c r="F33">
-        <v>15500</v>
-      </c>
-      <c r="G33">
-        <v>32364</v>
-      </c>
-      <c r="H33">
-        <v>992</v>
-      </c>
-      <c r="I33" t="str">
-        <v>28 Postes sources</v>
-      </c>
-      <c r="J33">
-        <v>93000</v>
-      </c>
-      <c r="K33" t="str">
-        <v>100% Sécurisé</v>
-      </c>
-      <c r="L33" t="str">
         <v>100% Validé</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L31"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1992,13 +1952,13 @@
         <v>Composante Soutirage Brut (CS)</v>
       </c>
       <c r="B2">
-        <v>312500</v>
+        <v>292500</v>
       </c>
       <c r="C2">
-        <v>70514</v>
+        <v>65724</v>
       </c>
       <c r="D2">
-        <v>241986</v>
+        <v>226776</v>
       </c>
     </row>
     <row r="3">
@@ -2006,13 +1966,13 @@
         <v>Composante Prix de Puissance Souscrite (PS)</v>
       </c>
       <c r="B3">
-        <v>185000</v>
+        <v>173000</v>
       </c>
       <c r="C3">
-        <v>124781</v>
+        <v>116563</v>
       </c>
       <c r="D3">
-        <v>60219</v>
+        <v>56437</v>
       </c>
     </row>
     <row r="4">
@@ -2020,13 +1980,13 @@
         <v>Pertes Réseau Non Récupérables (Limitation 1.5%)</v>
       </c>
       <c r="B4">
-        <v>128500</v>
+        <v>120250</v>
       </c>
       <c r="C4">
-        <v>38929</v>
+        <v>36337</v>
       </c>
       <c r="D4">
-        <v>89571</v>
+        <v>83913</v>
       </c>
     </row>
     <row r="5">
@@ -2034,13 +1994,13 @@
         <v>Composante Gestion &amp; Comptage (CG/CC)</v>
       </c>
       <c r="B5">
-        <v>71586</v>
+        <v>66684</v>
       </c>
       <c r="C5">
-        <v>22289</v>
+        <v>22503</v>
       </c>
       <c r="D5">
-        <v>49297</v>
+        <v>44181</v>
       </c>
     </row>
     <row r="6">
@@ -2048,13 +2008,13 @@
         <v>TOTAL FACTURE ANNUELLE RÉSEAU ENEDIS</v>
       </c>
       <c r="B6">
-        <v>697586</v>
+        <v>652434</v>
       </c>
       <c r="C6">
-        <v>257627</v>
+        <v>241127</v>
       </c>
       <c r="D6">
-        <v>439073</v>
+        <v>411307</v>
       </c>
     </row>
     <row r="8">
@@ -2062,7 +2022,7 @@
         <v>SYNTHÈSE DU GAIN SUR L'HORIZON 15 ANS</v>
       </c>
       <c r="B8" t="str">
-        <v>+ 6 586 095 € de marge additionnelle sécurisée pour les 31 stations</v>
+        <v>+ 6 169 605 € de marge additionnelle sécurisée pour les 29 stations</v>
       </c>
     </row>
   </sheetData>

</xml_diff>